<commit_message>
Actualizar plantillas: EquiArena, GranSuelo, LLP, Proctor
</commit_message>
<xml_diff>
--- a/app/templates/informes/EquiArena/Template_EquiArena.xlsx
+++ b/app/templates/informes/EquiArena/Template_EquiArena.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\EquiArena\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6764323F-BEE7-442D-9469-7EE07C96DA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AD288C-7B05-4AC5-9176-5DA14C381A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="556" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -845,7 +845,7 @@
     <t>-</t>
   </si>
   <si>
-    <t>Versión: 08 (11-06-2026)</t>
+    <t>Versión: 08 (12-06-2026)</t>
   </si>
 </sst>
 </file>
@@ -2945,6 +2945,123 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="178" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
@@ -2973,121 +3090,46 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="178" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3156,48 +3198,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -5773,36 +5773,36 @@
       <c r="N6" s="283"/>
     </row>
     <row r="7" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="437" t="s">
+      <c r="A7" s="409" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="437"/>
-      <c r="C7" s="437"/>
-      <c r="D7" s="437"/>
-      <c r="E7" s="437"/>
-      <c r="F7" s="437"/>
-      <c r="G7" s="437"/>
-      <c r="H7" s="437"/>
-      <c r="I7" s="437"/>
-      <c r="J7" s="437"/>
+      <c r="B7" s="409"/>
+      <c r="C7" s="409"/>
+      <c r="D7" s="409"/>
+      <c r="E7" s="409"/>
+      <c r="F7" s="409"/>
+      <c r="G7" s="409"/>
+      <c r="H7" s="409"/>
+      <c r="I7" s="409"/>
+      <c r="J7" s="409"/>
       <c r="M7" s="279" t="s">
         <v>119</v>
       </c>
       <c r="N7" s="283"/>
     </row>
     <row r="8" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="438" t="s">
+      <c r="A8" s="410" t="s">
         <v>122</v>
       </c>
-      <c r="B8" s="438"/>
-      <c r="C8" s="438"/>
-      <c r="D8" s="438"/>
-      <c r="E8" s="438"/>
-      <c r="F8" s="438"/>
-      <c r="G8" s="438"/>
-      <c r="H8" s="438"/>
-      <c r="I8" s="438"/>
-      <c r="J8" s="438"/>
+      <c r="B8" s="410"/>
+      <c r="C8" s="410"/>
+      <c r="D8" s="410"/>
+      <c r="E8" s="410"/>
+      <c r="F8" s="410"/>
+      <c r="G8" s="410"/>
+      <c r="H8" s="410"/>
+      <c r="I8" s="410"/>
+      <c r="J8" s="410"/>
       <c r="M8" s="279" t="s">
         <v>157</v>
       </c>
@@ -5825,22 +5825,22 @@
       <c r="N9" s="283"/>
     </row>
     <row r="10" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="439" t="s">
+      <c r="B10" s="411" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="439"/>
-      <c r="D10" s="439" t="s">
+      <c r="C10" s="411"/>
+      <c r="D10" s="411" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="439"/>
-      <c r="F10" s="439" t="s">
+      <c r="E10" s="411"/>
+      <c r="F10" s="411" t="s">
         <v>125</v>
       </c>
-      <c r="G10" s="439"/>
-      <c r="H10" s="439" t="s">
+      <c r="G10" s="411"/>
+      <c r="H10" s="411" t="s">
         <v>126</v>
       </c>
-      <c r="I10" s="439"/>
+      <c r="I10" s="411"/>
       <c r="J10" s="209"/>
       <c r="K10" s="210"/>
       <c r="L10" s="210"/>
@@ -5849,14 +5849,14 @@
     </row>
     <row r="11" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="211"/>
-      <c r="B11" s="439"/>
-      <c r="C11" s="439"/>
-      <c r="D11" s="439"/>
-      <c r="E11" s="439"/>
-      <c r="F11" s="439"/>
-      <c r="G11" s="439"/>
-      <c r="H11" s="439"/>
-      <c r="I11" s="439"/>
+      <c r="B11" s="411"/>
+      <c r="C11" s="411"/>
+      <c r="D11" s="411"/>
+      <c r="E11" s="411"/>
+      <c r="F11" s="411"/>
+      <c r="G11" s="411"/>
+      <c r="H11" s="411"/>
+      <c r="I11" s="411"/>
       <c r="J11" s="212"/>
       <c r="K11" s="210"/>
       <c r="L11" s="210"/>
@@ -5884,18 +5884,18 @@
       <c r="N12" s="284"/>
     </row>
     <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="440" t="s">
+      <c r="A13" s="412" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="441"/>
-      <c r="C13" s="441"/>
-      <c r="D13" s="441"/>
-      <c r="E13" s="441"/>
-      <c r="F13" s="441"/>
-      <c r="G13" s="441"/>
-      <c r="H13" s="441"/>
-      <c r="I13" s="441"/>
-      <c r="J13" s="442"/>
+      <c r="B13" s="413"/>
+      <c r="C13" s="413"/>
+      <c r="D13" s="413"/>
+      <c r="E13" s="413"/>
+      <c r="F13" s="413"/>
+      <c r="G13" s="413"/>
+      <c r="H13" s="413"/>
+      <c r="I13" s="413"/>
+      <c r="J13" s="414"/>
       <c r="K13" s="210"/>
       <c r="L13" s="210"/>
       <c r="M13" s="279" t="s">
@@ -5904,18 +5904,18 @@
       <c r="N13" s="284"/>
     </row>
     <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="434" t="s">
+      <c r="A14" s="406" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="435"/>
-      <c r="C14" s="435"/>
-      <c r="D14" s="435"/>
-      <c r="E14" s="435"/>
-      <c r="F14" s="435"/>
-      <c r="G14" s="435"/>
-      <c r="H14" s="435"/>
-      <c r="I14" s="435"/>
-      <c r="J14" s="436"/>
+      <c r="B14" s="407"/>
+      <c r="C14" s="407"/>
+      <c r="D14" s="407"/>
+      <c r="E14" s="407"/>
+      <c r="F14" s="407"/>
+      <c r="G14" s="407"/>
+      <c r="H14" s="407"/>
+      <c r="I14" s="407"/>
+      <c r="J14" s="408"/>
       <c r="K14" s="210"/>
       <c r="L14" s="210"/>
       <c r="M14" s="282"/>
@@ -5941,21 +5941,21 @@
     </row>
     <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="221"/>
-      <c r="B16" s="426" t="s">
+      <c r="B16" s="415" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="426"/>
-      <c r="D16" s="426"/>
+      <c r="C16" s="415"/>
+      <c r="D16" s="415"/>
       <c r="E16" s="222"/>
-      <c r="F16" s="427" t="s">
+      <c r="F16" s="416" t="s">
         <v>127</v>
       </c>
-      <c r="G16" s="427"/>
+      <c r="G16" s="416"/>
       <c r="H16" s="222"/>
-      <c r="I16" s="428" t="s">
+      <c r="I16" s="417" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="431"/>
+      <c r="J16" s="420"/>
       <c r="K16" s="210"/>
       <c r="L16" s="210"/>
       <c r="M16" s="279" t="s">
@@ -5965,15 +5965,15 @@
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="221"/>
-      <c r="B17" s="417"/>
-      <c r="C17" s="418"/>
-      <c r="D17" s="419"/>
+      <c r="B17" s="423"/>
+      <c r="C17" s="424"/>
+      <c r="D17" s="425"/>
       <c r="E17" s="223"/>
-      <c r="F17" s="417"/>
-      <c r="G17" s="419"/>
+      <c r="F17" s="423"/>
+      <c r="G17" s="425"/>
       <c r="H17" s="222"/>
-      <c r="I17" s="429"/>
-      <c r="J17" s="432"/>
+      <c r="I17" s="418"/>
+      <c r="J17" s="421"/>
       <c r="K17" s="210"/>
       <c r="L17" s="210"/>
       <c r="M17" s="279" t="s">
@@ -5986,8 +5986,8 @@
       <c r="F18" s="223"/>
       <c r="G18" s="223"/>
       <c r="H18" s="222"/>
-      <c r="I18" s="430"/>
-      <c r="J18" s="433"/>
+      <c r="I18" s="419"/>
+      <c r="J18" s="422"/>
       <c r="L18" s="210"/>
       <c r="M18" s="224"/>
     </row>
@@ -6007,11 +6007,11 @@
     </row>
     <row r="20" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="227"/>
-      <c r="B20" s="413" t="s">
+      <c r="B20" s="426" t="s">
         <v>129</v>
       </c>
-      <c r="C20" s="413"/>
-      <c r="D20" s="415"/>
+      <c r="C20" s="426"/>
+      <c r="D20" s="428"/>
       <c r="F20" s="229" t="s">
         <v>130</v>
       </c>
@@ -6024,12 +6024,12 @@
     </row>
     <row r="21" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="232"/>
-      <c r="B21" s="414"/>
-      <c r="C21" s="414"/>
-      <c r="D21" s="416"/>
-      <c r="F21" s="417"/>
-      <c r="G21" s="418"/>
-      <c r="H21" s="419"/>
+      <c r="B21" s="427"/>
+      <c r="C21" s="427"/>
+      <c r="D21" s="429"/>
+      <c r="F21" s="423"/>
+      <c r="G21" s="424"/>
+      <c r="H21" s="425"/>
       <c r="I21" s="230"/>
       <c r="J21" s="226"/>
       <c r="L21" s="231"/>
@@ -6303,11 +6303,11 @@
       <c r="G36" s="250" t="s">
         <v>1</v>
       </c>
-      <c r="H36" s="420">
+      <c r="H36" s="430">
         <v>31</v>
       </c>
-      <c r="I36" s="421"/>
-      <c r="J36" s="422"/>
+      <c r="I36" s="431"/>
+      <c r="J36" s="432"/>
       <c r="K36" s="210"/>
       <c r="L36" s="210"/>
     </row>
@@ -6326,15 +6326,15 @@
       <c r="L37" s="210"/>
     </row>
     <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="423" t="s">
+      <c r="A38" s="433" t="s">
         <v>146</v>
       </c>
-      <c r="B38" s="424"/>
-      <c r="C38" s="425"/>
-      <c r="D38" s="423" t="s">
+      <c r="B38" s="434"/>
+      <c r="C38" s="435"/>
+      <c r="D38" s="433" t="s">
         <v>147</v>
       </c>
-      <c r="E38" s="425"/>
+      <c r="E38" s="435"/>
       <c r="F38" s="271" t="s">
         <v>100</v>
       </c>
@@ -6346,13 +6346,13 @@
       <c r="L38" s="210"/>
     </row>
     <row r="39" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="406" t="s">
+      <c r="A39" s="436" t="s">
         <v>148</v>
       </c>
-      <c r="B39" s="407"/>
-      <c r="C39" s="408"/>
-      <c r="D39" s="406"/>
-      <c r="E39" s="408"/>
+      <c r="B39" s="437"/>
+      <c r="C39" s="438"/>
+      <c r="D39" s="436"/>
+      <c r="E39" s="438"/>
       <c r="F39" s="233"/>
       <c r="G39" s="234"/>
       <c r="H39" s="234"/>
@@ -6362,13 +6362,13 @@
       <c r="L39" s="210"/>
     </row>
     <row r="40" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="406" t="s">
+      <c r="A40" s="436" t="s">
         <v>149</v>
       </c>
-      <c r="B40" s="407"/>
-      <c r="C40" s="408"/>
-      <c r="D40" s="406"/>
-      <c r="E40" s="408"/>
+      <c r="B40" s="437"/>
+      <c r="C40" s="438"/>
+      <c r="D40" s="436"/>
+      <c r="E40" s="438"/>
       <c r="F40" s="274"/>
       <c r="G40" s="272"/>
       <c r="H40" s="272"/>
@@ -6378,61 +6378,61 @@
       <c r="L40" s="210"/>
     </row>
     <row r="41" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="406" t="s">
+      <c r="A41" s="436" t="s">
         <v>150</v>
       </c>
-      <c r="B41" s="407"/>
-      <c r="C41" s="408"/>
-      <c r="D41" s="406"/>
-      <c r="E41" s="408"/>
+      <c r="B41" s="437"/>
+      <c r="C41" s="438"/>
+      <c r="D41" s="436"/>
+      <c r="E41" s="438"/>
       <c r="F41" s="221"/>
       <c r="K41" s="210"/>
       <c r="L41" s="210"/>
     </row>
     <row r="42" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="410" t="s">
+      <c r="A42" s="440" t="s">
         <v>151</v>
       </c>
-      <c r="B42" s="411"/>
-      <c r="C42" s="412"/>
-      <c r="D42" s="406"/>
-      <c r="E42" s="408"/>
+      <c r="B42" s="441"/>
+      <c r="C42" s="442"/>
+      <c r="D42" s="436"/>
+      <c r="E42" s="438"/>
       <c r="F42" s="221"/>
       <c r="K42" s="210"/>
       <c r="L42" s="210"/>
     </row>
     <row r="43" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="410" t="s">
+      <c r="A43" s="440" t="s">
         <v>152</v>
       </c>
-      <c r="B43" s="411"/>
-      <c r="C43" s="412"/>
-      <c r="D43" s="406"/>
-      <c r="E43" s="408"/>
+      <c r="B43" s="441"/>
+      <c r="C43" s="442"/>
+      <c r="D43" s="436"/>
+      <c r="E43" s="438"/>
       <c r="F43" s="221"/>
       <c r="K43" s="210"/>
       <c r="L43" s="210"/>
     </row>
     <row r="44" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="406" t="s">
+      <c r="A44" s="436" t="s">
         <v>153</v>
       </c>
-      <c r="B44" s="407"/>
-      <c r="C44" s="408"/>
-      <c r="D44" s="406"/>
-      <c r="E44" s="408"/>
+      <c r="B44" s="437"/>
+      <c r="C44" s="438"/>
+      <c r="D44" s="436"/>
+      <c r="E44" s="438"/>
       <c r="F44" s="221"/>
       <c r="K44" s="210"/>
       <c r="L44" s="210"/>
     </row>
     <row r="45" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="406" t="s">
+      <c r="A45" s="436" t="s">
         <v>154</v>
       </c>
-      <c r="B45" s="407"/>
-      <c r="C45" s="408"/>
-      <c r="D45" s="406"/>
-      <c r="E45" s="408"/>
+      <c r="B45" s="437"/>
+      <c r="C45" s="438"/>
+      <c r="D45" s="436"/>
+      <c r="E45" s="438"/>
       <c r="F45" s="221"/>
       <c r="K45" s="210"/>
       <c r="L45" s="210"/>
@@ -6525,18 +6525,18 @@
     </row>
     <row r="53" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="409" t="s">
+      <c r="A54" s="439" t="s">
         <v>170</v>
       </c>
-      <c r="B54" s="409"/>
-      <c r="C54" s="409"/>
-      <c r="D54" s="409"/>
-      <c r="E54" s="409"/>
-      <c r="F54" s="409"/>
-      <c r="G54" s="409"/>
-      <c r="H54" s="409"/>
-      <c r="I54" s="409"/>
-      <c r="J54" s="409"/>
+      <c r="B54" s="439"/>
+      <c r="C54" s="439"/>
+      <c r="D54" s="439"/>
+      <c r="E54" s="439"/>
+      <c r="F54" s="439"/>
+      <c r="G54" s="439"/>
+      <c r="H54" s="439"/>
+      <c r="I54" s="439"/>
+      <c r="J54" s="439"/>
     </row>
     <row r="55" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6548,6 +6548,33 @@
     <protectedRange sqref="H31:J31" name="Rango8_1"/>
   </protectedRanges>
   <mergeCells count="39">
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A54:J54"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J16:J18"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="A7:J7"/>
     <mergeCell ref="A8:J8"/>
@@ -6560,33 +6587,6 @@
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="A13:J13"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="J16:J18"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="B20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A54:J54"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0" bottom="0" header="0" footer="0"/>
@@ -6637,38 +6637,38 @@
       <c r="M1" s="295"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="464" t="s">
+      <c r="A2" s="443" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="464"/>
-      <c r="C2" s="464"/>
-      <c r="D2" s="464"/>
-      <c r="E2" s="464"/>
-      <c r="F2" s="464"/>
-      <c r="G2" s="464"/>
-      <c r="H2" s="464"/>
-      <c r="I2" s="464"/>
-      <c r="J2" s="464"/>
-      <c r="K2" s="464"/>
-      <c r="L2" s="464"/>
-      <c r="M2" s="464"/>
+      <c r="B2" s="443"/>
+      <c r="C2" s="443"/>
+      <c r="D2" s="443"/>
+      <c r="E2" s="443"/>
+      <c r="F2" s="443"/>
+      <c r="G2" s="443"/>
+      <c r="H2" s="443"/>
+      <c r="I2" s="443"/>
+      <c r="J2" s="443"/>
+      <c r="K2" s="443"/>
+      <c r="L2" s="443"/>
+      <c r="M2" s="443"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="465">
+      <c r="A3" s="444">
         <v>0</v>
       </c>
-      <c r="B3" s="465"/>
-      <c r="C3" s="465"/>
-      <c r="D3" s="465"/>
-      <c r="E3" s="465"/>
-      <c r="F3" s="465"/>
-      <c r="G3" s="465"/>
-      <c r="H3" s="465"/>
-      <c r="I3" s="465"/>
-      <c r="J3" s="465"/>
-      <c r="K3" s="465"/>
-      <c r="L3" s="465"/>
-      <c r="M3" s="465"/>
+      <c r="B3" s="444"/>
+      <c r="C3" s="444"/>
+      <c r="D3" s="444"/>
+      <c r="E3" s="444"/>
+      <c r="F3" s="444"/>
+      <c r="G3" s="444"/>
+      <c r="H3" s="444"/>
+      <c r="I3" s="444"/>
+      <c r="J3" s="444"/>
+      <c r="K3" s="444"/>
+      <c r="L3" s="444"/>
+      <c r="M3" s="444"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6678,17 +6678,17 @@
       <c r="B5" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="476">
+      <c r="C5" s="455">
         <f>+FORMATO!N2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="476"/>
-      <c r="E5" s="476"/>
-      <c r="F5" s="476"/>
-      <c r="G5" s="476"/>
-      <c r="H5" s="476"/>
-      <c r="I5" s="476"/>
-      <c r="J5" s="476"/>
+      <c r="D5" s="455"/>
+      <c r="E5" s="455"/>
+      <c r="F5" s="455"/>
+      <c r="G5" s="455"/>
+      <c r="H5" s="455"/>
+      <c r="I5" s="455"/>
+      <c r="J5" s="455"/>
       <c r="K5" s="299" t="s">
         <v>20</v>
       </c>
@@ -6706,17 +6706,17 @@
       <c r="B6" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="476">
+      <c r="C6" s="455">
         <f>+FORMATO!N3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="476"/>
-      <c r="E6" s="476"/>
-      <c r="F6" s="476"/>
-      <c r="G6" s="476"/>
-      <c r="H6" s="476"/>
-      <c r="I6" s="476"/>
-      <c r="J6" s="476"/>
+      <c r="D6" s="455"/>
+      <c r="E6" s="455"/>
+      <c r="F6" s="455"/>
+      <c r="G6" s="455"/>
+      <c r="H6" s="455"/>
+      <c r="I6" s="455"/>
+      <c r="J6" s="455"/>
       <c r="K6" s="279" t="s">
         <v>119</v>
       </c>
@@ -6738,17 +6738,17 @@
       <c r="B7" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="476">
+      <c r="C7" s="455">
         <f>+FORMATO!N4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="476"/>
-      <c r="E7" s="476"/>
-      <c r="F7" s="476"/>
-      <c r="G7" s="476"/>
-      <c r="H7" s="476"/>
-      <c r="I7" s="476"/>
-      <c r="J7" s="476"/>
+      <c r="D7" s="455"/>
+      <c r="E7" s="455"/>
+      <c r="F7" s="455"/>
+      <c r="G7" s="455"/>
+      <c r="H7" s="455"/>
+      <c r="I7" s="455"/>
+      <c r="J7" s="455"/>
       <c r="K7" s="279" t="s">
         <v>158</v>
       </c>
@@ -6770,17 +6770,17 @@
       <c r="B8" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="476">
+      <c r="C8" s="455">
         <f>+FORMATO!N5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="476"/>
-      <c r="E8" s="476"/>
-      <c r="F8" s="476"/>
-      <c r="G8" s="476"/>
-      <c r="H8" s="476"/>
-      <c r="I8" s="476"/>
-      <c r="J8" s="476"/>
+      <c r="D8" s="455"/>
+      <c r="E8" s="455"/>
+      <c r="F8" s="455"/>
+      <c r="G8" s="455"/>
+      <c r="H8" s="455"/>
+      <c r="I8" s="455"/>
+      <c r="J8" s="455"/>
       <c r="K8" s="304" t="s">
         <v>36</v>
       </c>
@@ -6816,41 +6816,41 @@
       <c r="P9" s="303"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="468" t="s">
+      <c r="A10" s="447" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="469"/>
-      <c r="C10" s="469"/>
-      <c r="D10" s="469"/>
-      <c r="E10" s="469"/>
-      <c r="F10" s="469"/>
-      <c r="G10" s="469"/>
-      <c r="H10" s="469"/>
-      <c r="I10" s="469"/>
-      <c r="J10" s="469"/>
-      <c r="K10" s="469"/>
-      <c r="L10" s="469"/>
-      <c r="M10" s="470"/>
+      <c r="B10" s="448"/>
+      <c r="C10" s="448"/>
+      <c r="D10" s="448"/>
+      <c r="E10" s="448"/>
+      <c r="F10" s="448"/>
+      <c r="G10" s="448"/>
+      <c r="H10" s="448"/>
+      <c r="I10" s="448"/>
+      <c r="J10" s="448"/>
+      <c r="K10" s="448"/>
+      <c r="L10" s="448"/>
+      <c r="M10" s="449"/>
       <c r="N10" s="303"/>
       <c r="O10" s="303"/>
       <c r="P10" s="303"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="471" t="s">
+      <c r="A11" s="450" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="472"/>
-      <c r="C11" s="472"/>
-      <c r="D11" s="472"/>
-      <c r="E11" s="472"/>
-      <c r="F11" s="472"/>
-      <c r="G11" s="472"/>
-      <c r="H11" s="472"/>
-      <c r="I11" s="472"/>
-      <c r="J11" s="472"/>
-      <c r="K11" s="472"/>
-      <c r="L11" s="472"/>
-      <c r="M11" s="473"/>
+      <c r="B11" s="451"/>
+      <c r="C11" s="451"/>
+      <c r="D11" s="451"/>
+      <c r="E11" s="451"/>
+      <c r="F11" s="451"/>
+      <c r="G11" s="451"/>
+      <c r="H11" s="451"/>
+      <c r="I11" s="451"/>
+      <c r="J11" s="451"/>
+      <c r="K11" s="451"/>
+      <c r="L11" s="451"/>
+      <c r="M11" s="452"/>
       <c r="N11" s="303"/>
       <c r="O11" s="303"/>
       <c r="P11" s="303"/>
@@ -6874,13 +6874,13 @@
       <c r="P12" s="303"/>
     </row>
     <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="474" t="s">
+      <c r="A13" s="453" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="475"/>
-      <c r="C13" s="475"/>
-      <c r="D13" s="475"/>
-      <c r="E13" s="475"/>
+      <c r="B13" s="454"/>
+      <c r="C13" s="454"/>
+      <c r="D13" s="454"/>
+      <c r="E13" s="454"/>
       <c r="F13" s="318"/>
       <c r="G13" s="318"/>
       <c r="H13" s="318"/>
@@ -7011,15 +7011,15 @@
       <c r="A18" s="341"/>
       <c r="B18" s="342"/>
       <c r="C18" s="342"/>
-      <c r="D18" s="466"/>
-      <c r="E18" s="466"/>
+      <c r="D18" s="445"/>
+      <c r="E18" s="445"/>
       <c r="F18" s="342"/>
       <c r="G18" s="342"/>
       <c r="H18" s="342"/>
       <c r="I18" s="343"/>
       <c r="J18" s="343"/>
-      <c r="K18" s="467"/>
-      <c r="L18" s="467"/>
+      <c r="K18" s="446"/>
+      <c r="L18" s="446"/>
       <c r="M18" s="344"/>
       <c r="N18" s="303"/>
       <c r="O18" s="345"/>
@@ -7029,18 +7029,18 @@
       <c r="A19" s="346"/>
       <c r="B19" s="347"/>
       <c r="C19" s="347"/>
-      <c r="D19" s="443" t="s">
+      <c r="D19" s="456" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="444"/>
-      <c r="F19" s="444"/>
-      <c r="G19" s="444"/>
-      <c r="H19" s="445"/>
-      <c r="I19" s="461" t="s">
+      <c r="E19" s="457"/>
+      <c r="F19" s="457"/>
+      <c r="G19" s="457"/>
+      <c r="H19" s="458"/>
+      <c r="I19" s="474" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="461"/>
-      <c r="K19" s="462"/>
+      <c r="J19" s="474"/>
+      <c r="K19" s="475"/>
       <c r="L19" s="348"/>
       <c r="M19" s="349"/>
       <c r="N19" s="303"/>
@@ -7051,11 +7051,11 @@
       <c r="A20" s="350"/>
       <c r="B20" s="295"/>
       <c r="C20" s="295"/>
-      <c r="D20" s="446"/>
-      <c r="E20" s="447"/>
-      <c r="F20" s="447"/>
-      <c r="G20" s="447"/>
-      <c r="H20" s="448"/>
+      <c r="D20" s="459"/>
+      <c r="E20" s="460"/>
+      <c r="F20" s="460"/>
+      <c r="G20" s="460"/>
+      <c r="H20" s="461"/>
       <c r="I20" s="351">
         <v>1</v>
       </c>
@@ -7127,8 +7127,8 @@
         <f>+Datos!I14</f>
         <v>0</v>
       </c>
-      <c r="L22" s="455"/>
-      <c r="M22" s="454"/>
+      <c r="L22" s="468"/>
+      <c r="M22" s="467"/>
       <c r="N22" s="303"/>
       <c r="O22" s="364"/>
       <c r="P22" s="303"/>
@@ -7158,8 +7158,8 @@
         <f>+Datos!I15</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L23" s="453"/>
-      <c r="M23" s="454"/>
+      <c r="L23" s="466"/>
+      <c r="M23" s="467"/>
       <c r="N23" s="303"/>
       <c r="O23" s="303"/>
       <c r="P23" s="364"/>
@@ -7177,12 +7177,12 @@
       <c r="H24" s="360" t="s">
         <v>1</v>
       </c>
-      <c r="I24" s="456" t="e">
+      <c r="I24" s="469" t="e">
         <f>+Datos!G16</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J24" s="457"/>
-      <c r="K24" s="458"/>
+      <c r="J24" s="470"/>
+      <c r="K24" s="471"/>
       <c r="L24" s="369"/>
       <c r="M24" s="362"/>
       <c r="N24" s="303"/>
@@ -7244,10 +7244,10 @@
       <c r="C28" s="386"/>
       <c r="D28" s="367"/>
       <c r="E28" s="369"/>
-      <c r="F28" s="459" t="s">
+      <c r="F28" s="472" t="s">
         <v>176</v>
       </c>
-      <c r="G28" s="460"/>
+      <c r="G28" s="473"/>
       <c r="M28" s="384"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -7270,11 +7270,11 @@
       <c r="C30" s="386"/>
       <c r="D30" s="367"/>
       <c r="E30" s="369"/>
-      <c r="F30" s="449">
+      <c r="F30" s="462">
         <f>+Datos!E25</f>
         <v>0</v>
       </c>
-      <c r="G30" s="450"/>
+      <c r="G30" s="463"/>
       <c r="M30" s="384"/>
     </row>
     <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7285,11 +7285,11 @@
       <c r="C31" s="386"/>
       <c r="D31" s="367"/>
       <c r="E31" s="369"/>
-      <c r="F31" s="449">
+      <c r="F31" s="462">
         <f>+Datos!E26</f>
         <v>0</v>
       </c>
-      <c r="G31" s="450"/>
+      <c r="G31" s="463"/>
       <c r="M31" s="384"/>
     </row>
     <row r="32" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7326,95 +7326,95 @@
       <c r="M34" s="393"/>
     </row>
     <row r="35" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="463" t="s">
+      <c r="A35" s="476" t="s">
         <v>171</v>
       </c>
-      <c r="B35" s="463"/>
-      <c r="C35" s="463"/>
-      <c r="D35" s="463"/>
-      <c r="E35" s="463"/>
-      <c r="F35" s="463"/>
-      <c r="G35" s="463"/>
-      <c r="H35" s="463"/>
-      <c r="I35" s="463"/>
-      <c r="J35" s="463"/>
-      <c r="K35" s="463"/>
-      <c r="L35" s="463"/>
-      <c r="M35" s="463"/>
+      <c r="B35" s="476"/>
+      <c r="C35" s="476"/>
+      <c r="D35" s="476"/>
+      <c r="E35" s="476"/>
+      <c r="F35" s="476"/>
+      <c r="G35" s="476"/>
+      <c r="H35" s="476"/>
+      <c r="I35" s="476"/>
+      <c r="J35" s="476"/>
+      <c r="K35" s="476"/>
+      <c r="L35" s="476"/>
+      <c r="M35" s="476"/>
     </row>
     <row r="36" spans="1:16" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="452" t="s">
+      <c r="A36" s="465" t="s">
         <v>172</v>
       </c>
-      <c r="B36" s="452"/>
-      <c r="C36" s="452"/>
-      <c r="D36" s="452"/>
-      <c r="E36" s="452"/>
-      <c r="F36" s="452"/>
-      <c r="G36" s="452"/>
-      <c r="H36" s="452"/>
-      <c r="I36" s="452"/>
-      <c r="J36" s="452"/>
-      <c r="K36" s="452"/>
-      <c r="L36" s="452"/>
-      <c r="M36" s="452"/>
+      <c r="B36" s="465"/>
+      <c r="C36" s="465"/>
+      <c r="D36" s="465"/>
+      <c r="E36" s="465"/>
+      <c r="F36" s="465"/>
+      <c r="G36" s="465"/>
+      <c r="H36" s="465"/>
+      <c r="I36" s="465"/>
+      <c r="J36" s="465"/>
+      <c r="K36" s="465"/>
+      <c r="L36" s="465"/>
+      <c r="M36" s="465"/>
     </row>
     <row r="37" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="452" t="s">
+      <c r="A37" s="465" t="s">
         <v>173</v>
       </c>
-      <c r="B37" s="452"/>
-      <c r="C37" s="452"/>
-      <c r="D37" s="452"/>
-      <c r="E37" s="452"/>
-      <c r="F37" s="452"/>
-      <c r="G37" s="452"/>
-      <c r="H37" s="452"/>
-      <c r="I37" s="452"/>
-      <c r="J37" s="452"/>
-      <c r="K37" s="452"/>
-      <c r="L37" s="452"/>
-      <c r="M37" s="452"/>
+      <c r="B37" s="465"/>
+      <c r="C37" s="465"/>
+      <c r="D37" s="465"/>
+      <c r="E37" s="465"/>
+      <c r="F37" s="465"/>
+      <c r="G37" s="465"/>
+      <c r="H37" s="465"/>
+      <c r="I37" s="465"/>
+      <c r="J37" s="465"/>
+      <c r="K37" s="465"/>
+      <c r="L37" s="465"/>
+      <c r="M37" s="465"/>
       <c r="N37" s="303"/>
       <c r="O37" s="303"/>
       <c r="P37" s="303"/>
     </row>
     <row r="38" spans="1:16" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="452" t="s">
+      <c r="A38" s="465" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="452"/>
-      <c r="C38" s="452"/>
-      <c r="D38" s="452"/>
-      <c r="E38" s="452"/>
-      <c r="F38" s="452"/>
-      <c r="G38" s="452"/>
-      <c r="H38" s="452"/>
-      <c r="I38" s="452"/>
-      <c r="J38" s="452"/>
-      <c r="K38" s="452"/>
-      <c r="L38" s="452"/>
-      <c r="M38" s="452"/>
+      <c r="B38" s="465"/>
+      <c r="C38" s="465"/>
+      <c r="D38" s="465"/>
+      <c r="E38" s="465"/>
+      <c r="F38" s="465"/>
+      <c r="G38" s="465"/>
+      <c r="H38" s="465"/>
+      <c r="I38" s="465"/>
+      <c r="J38" s="465"/>
+      <c r="K38" s="465"/>
+      <c r="L38" s="465"/>
+      <c r="M38" s="465"/>
       <c r="N38" s="303"/>
       <c r="O38" s="303"/>
       <c r="P38" s="303"/>
     </row>
     <row r="39" spans="1:16" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="451" t="s">
+      <c r="A39" s="464" t="s">
         <v>175</v>
       </c>
-      <c r="B39" s="451"/>
-      <c r="C39" s="451"/>
-      <c r="D39" s="451"/>
-      <c r="E39" s="451"/>
-      <c r="F39" s="451"/>
-      <c r="G39" s="451"/>
-      <c r="H39" s="451"/>
-      <c r="I39" s="451"/>
-      <c r="J39" s="451"/>
-      <c r="K39" s="451"/>
-      <c r="L39" s="451"/>
-      <c r="M39" s="451"/>
+      <c r="B39" s="464"/>
+      <c r="C39" s="464"/>
+      <c r="D39" s="464"/>
+      <c r="E39" s="464"/>
+      <c r="F39" s="464"/>
+      <c r="G39" s="464"/>
+      <c r="H39" s="464"/>
+      <c r="I39" s="464"/>
+      <c r="J39" s="464"/>
+      <c r="K39" s="464"/>
+      <c r="L39" s="464"/>
+      <c r="M39" s="464"/>
       <c r="N39" s="303"/>
       <c r="O39" s="303"/>
       <c r="P39" s="303"/>
@@ -7619,17 +7619,6 @@
     <protectedRange sqref="C5:E6" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="24">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:M11"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="C6:J6"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C8:J8"/>
     <mergeCell ref="D19:H20"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F31:G31"/>
@@ -7643,6 +7632,17 @@
     <mergeCell ref="A35:M35"/>
     <mergeCell ref="A36:M36"/>
     <mergeCell ref="A38:M38"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C8:J8"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F28:G28" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>

<commit_message>
chore: update Excel templates and backup previous versions
</commit_message>
<xml_diff>
--- a/app/templates/informes/EquiArena/Template_EquiArena.xlsx
+++ b/app/templates/informes/EquiArena/Template_EquiArena.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\EquiArena\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.1 Informe Suelo\INFORME ACREDITADO-E ISO\6.1 JUNIO INICIA 15-06-25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AD288C-7B05-4AC5-9176-5DA14C381A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{539911C6-48A8-4690-B9CD-F42F5202E243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="556" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2945,6 +2945,115 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="1"/>
@@ -2981,114 +3090,72 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="44" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3131,73 +3198,6 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3596,7 +3596,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-PE"/>
+            <a:endParaRPr lang="es-ES"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="119672192"/>
@@ -3633,7 +3633,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-PE"/>
+            <a:endParaRPr lang="es-ES"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="119670272"/>
@@ -3672,7 +3672,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-PE"/>
+      <a:endParaRPr lang="es-ES"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4648,7 +4648,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4707,7 +4707,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="datos de ecuacion del anillo"/>
@@ -4826,7 +4826,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4877,7 +4877,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4929,7 +4929,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BGA"/>
@@ -4961,7 +4961,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -5773,36 +5773,36 @@
       <c r="N6" s="283"/>
     </row>
     <row r="7" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="409" t="s">
+      <c r="A7" s="437" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="409"/>
-      <c r="C7" s="409"/>
-      <c r="D7" s="409"/>
-      <c r="E7" s="409"/>
-      <c r="F7" s="409"/>
-      <c r="G7" s="409"/>
-      <c r="H7" s="409"/>
-      <c r="I7" s="409"/>
-      <c r="J7" s="409"/>
+      <c r="B7" s="437"/>
+      <c r="C7" s="437"/>
+      <c r="D7" s="437"/>
+      <c r="E7" s="437"/>
+      <c r="F7" s="437"/>
+      <c r="G7" s="437"/>
+      <c r="H7" s="437"/>
+      <c r="I7" s="437"/>
+      <c r="J7" s="437"/>
       <c r="M7" s="279" t="s">
         <v>119</v>
       </c>
       <c r="N7" s="283"/>
     </row>
     <row r="8" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="410" t="s">
+      <c r="A8" s="438" t="s">
         <v>122</v>
       </c>
-      <c r="B8" s="410"/>
-      <c r="C8" s="410"/>
-      <c r="D8" s="410"/>
-      <c r="E8" s="410"/>
-      <c r="F8" s="410"/>
-      <c r="G8" s="410"/>
-      <c r="H8" s="410"/>
-      <c r="I8" s="410"/>
-      <c r="J8" s="410"/>
+      <c r="B8" s="438"/>
+      <c r="C8" s="438"/>
+      <c r="D8" s="438"/>
+      <c r="E8" s="438"/>
+      <c r="F8" s="438"/>
+      <c r="G8" s="438"/>
+      <c r="H8" s="438"/>
+      <c r="I8" s="438"/>
+      <c r="J8" s="438"/>
       <c r="M8" s="279" t="s">
         <v>157</v>
       </c>
@@ -5825,22 +5825,22 @@
       <c r="N9" s="283"/>
     </row>
     <row r="10" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="411" t="s">
+      <c r="B10" s="439" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="411"/>
-      <c r="D10" s="411" t="s">
+      <c r="C10" s="439"/>
+      <c r="D10" s="439" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="411"/>
-      <c r="F10" s="411" t="s">
+      <c r="E10" s="439"/>
+      <c r="F10" s="439" t="s">
         <v>125</v>
       </c>
-      <c r="G10" s="411"/>
-      <c r="H10" s="411" t="s">
+      <c r="G10" s="439"/>
+      <c r="H10" s="439" t="s">
         <v>126</v>
       </c>
-      <c r="I10" s="411"/>
+      <c r="I10" s="439"/>
       <c r="J10" s="209"/>
       <c r="K10" s="210"/>
       <c r="L10" s="210"/>
@@ -5849,14 +5849,14 @@
     </row>
     <row r="11" spans="1:14" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="211"/>
-      <c r="B11" s="411"/>
-      <c r="C11" s="411"/>
-      <c r="D11" s="411"/>
-      <c r="E11" s="411"/>
-      <c r="F11" s="411"/>
-      <c r="G11" s="411"/>
-      <c r="H11" s="411"/>
-      <c r="I11" s="411"/>
+      <c r="B11" s="439"/>
+      <c r="C11" s="439"/>
+      <c r="D11" s="439"/>
+      <c r="E11" s="439"/>
+      <c r="F11" s="439"/>
+      <c r="G11" s="439"/>
+      <c r="H11" s="439"/>
+      <c r="I11" s="439"/>
       <c r="J11" s="212"/>
       <c r="K11" s="210"/>
       <c r="L11" s="210"/>
@@ -5884,18 +5884,18 @@
       <c r="N12" s="284"/>
     </row>
     <row r="13" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="412" t="s">
+      <c r="A13" s="440" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="413"/>
-      <c r="C13" s="413"/>
-      <c r="D13" s="413"/>
-      <c r="E13" s="413"/>
-      <c r="F13" s="413"/>
-      <c r="G13" s="413"/>
-      <c r="H13" s="413"/>
-      <c r="I13" s="413"/>
-      <c r="J13" s="414"/>
+      <c r="B13" s="441"/>
+      <c r="C13" s="441"/>
+      <c r="D13" s="441"/>
+      <c r="E13" s="441"/>
+      <c r="F13" s="441"/>
+      <c r="G13" s="441"/>
+      <c r="H13" s="441"/>
+      <c r="I13" s="441"/>
+      <c r="J13" s="442"/>
       <c r="K13" s="210"/>
       <c r="L13" s="210"/>
       <c r="M13" s="279" t="s">
@@ -5904,18 +5904,18 @@
       <c r="N13" s="284"/>
     </row>
     <row r="14" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="406" t="s">
+      <c r="A14" s="434" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="407"/>
-      <c r="C14" s="407"/>
-      <c r="D14" s="407"/>
-      <c r="E14" s="407"/>
-      <c r="F14" s="407"/>
-      <c r="G14" s="407"/>
-      <c r="H14" s="407"/>
-      <c r="I14" s="407"/>
-      <c r="J14" s="408"/>
+      <c r="B14" s="435"/>
+      <c r="C14" s="435"/>
+      <c r="D14" s="435"/>
+      <c r="E14" s="435"/>
+      <c r="F14" s="435"/>
+      <c r="G14" s="435"/>
+      <c r="H14" s="435"/>
+      <c r="I14" s="435"/>
+      <c r="J14" s="436"/>
       <c r="K14" s="210"/>
       <c r="L14" s="210"/>
       <c r="M14" s="282"/>
@@ -5941,21 +5941,21 @@
     </row>
     <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="221"/>
-      <c r="B16" s="415" t="s">
+      <c r="B16" s="426" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="415"/>
-      <c r="D16" s="415"/>
+      <c r="C16" s="426"/>
+      <c r="D16" s="426"/>
       <c r="E16" s="222"/>
-      <c r="F16" s="416" t="s">
+      <c r="F16" s="427" t="s">
         <v>127</v>
       </c>
-      <c r="G16" s="416"/>
+      <c r="G16" s="427"/>
       <c r="H16" s="222"/>
-      <c r="I16" s="417" t="s">
+      <c r="I16" s="428" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="420"/>
+      <c r="J16" s="431"/>
       <c r="K16" s="210"/>
       <c r="L16" s="210"/>
       <c r="M16" s="279" t="s">
@@ -5965,15 +5965,15 @@
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="221"/>
-      <c r="B17" s="423"/>
-      <c r="C17" s="424"/>
-      <c r="D17" s="425"/>
+      <c r="B17" s="417"/>
+      <c r="C17" s="418"/>
+      <c r="D17" s="419"/>
       <c r="E17" s="223"/>
-      <c r="F17" s="423"/>
-      <c r="G17" s="425"/>
+      <c r="F17" s="417"/>
+      <c r="G17" s="419"/>
       <c r="H17" s="222"/>
-      <c r="I17" s="418"/>
-      <c r="J17" s="421"/>
+      <c r="I17" s="429"/>
+      <c r="J17" s="432"/>
       <c r="K17" s="210"/>
       <c r="L17" s="210"/>
       <c r="M17" s="279" t="s">
@@ -5986,8 +5986,8 @@
       <c r="F18" s="223"/>
       <c r="G18" s="223"/>
       <c r="H18" s="222"/>
-      <c r="I18" s="419"/>
-      <c r="J18" s="422"/>
+      <c r="I18" s="430"/>
+      <c r="J18" s="433"/>
       <c r="L18" s="210"/>
       <c r="M18" s="224"/>
     </row>
@@ -6007,11 +6007,11 @@
     </row>
     <row r="20" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="227"/>
-      <c r="B20" s="426" t="s">
+      <c r="B20" s="413" t="s">
         <v>129</v>
       </c>
-      <c r="C20" s="426"/>
-      <c r="D20" s="428"/>
+      <c r="C20" s="413"/>
+      <c r="D20" s="415"/>
       <c r="F20" s="229" t="s">
         <v>130</v>
       </c>
@@ -6024,12 +6024,12 @@
     </row>
     <row r="21" spans="1:14" s="228" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="232"/>
-      <c r="B21" s="427"/>
-      <c r="C21" s="427"/>
-      <c r="D21" s="429"/>
-      <c r="F21" s="423"/>
-      <c r="G21" s="424"/>
-      <c r="H21" s="425"/>
+      <c r="B21" s="414"/>
+      <c r="C21" s="414"/>
+      <c r="D21" s="416"/>
+      <c r="F21" s="417"/>
+      <c r="G21" s="418"/>
+      <c r="H21" s="419"/>
       <c r="I21" s="230"/>
       <c r="J21" s="226"/>
       <c r="L21" s="231"/>
@@ -6303,11 +6303,11 @@
       <c r="G36" s="250" t="s">
         <v>1</v>
       </c>
-      <c r="H36" s="430">
+      <c r="H36" s="420">
         <v>31</v>
       </c>
-      <c r="I36" s="431"/>
-      <c r="J36" s="432"/>
+      <c r="I36" s="421"/>
+      <c r="J36" s="422"/>
       <c r="K36" s="210"/>
       <c r="L36" s="210"/>
     </row>
@@ -6326,15 +6326,15 @@
       <c r="L37" s="210"/>
     </row>
     <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="433" t="s">
+      <c r="A38" s="423" t="s">
         <v>146</v>
       </c>
-      <c r="B38" s="434"/>
-      <c r="C38" s="435"/>
-      <c r="D38" s="433" t="s">
+      <c r="B38" s="424"/>
+      <c r="C38" s="425"/>
+      <c r="D38" s="423" t="s">
         <v>147</v>
       </c>
-      <c r="E38" s="435"/>
+      <c r="E38" s="425"/>
       <c r="F38" s="271" t="s">
         <v>100</v>
       </c>
@@ -6346,13 +6346,13 @@
       <c r="L38" s="210"/>
     </row>
     <row r="39" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="436" t="s">
+      <c r="A39" s="406" t="s">
         <v>148</v>
       </c>
-      <c r="B39" s="437"/>
-      <c r="C39" s="438"/>
-      <c r="D39" s="436"/>
-      <c r="E39" s="438"/>
+      <c r="B39" s="407"/>
+      <c r="C39" s="408"/>
+      <c r="D39" s="406"/>
+      <c r="E39" s="408"/>
       <c r="F39" s="233"/>
       <c r="G39" s="234"/>
       <c r="H39" s="234"/>
@@ -6362,13 +6362,13 @@
       <c r="L39" s="210"/>
     </row>
     <row r="40" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="436" t="s">
+      <c r="A40" s="406" t="s">
         <v>149</v>
       </c>
-      <c r="B40" s="437"/>
-      <c r="C40" s="438"/>
-      <c r="D40" s="436"/>
-      <c r="E40" s="438"/>
+      <c r="B40" s="407"/>
+      <c r="C40" s="408"/>
+      <c r="D40" s="406"/>
+      <c r="E40" s="408"/>
       <c r="F40" s="274"/>
       <c r="G40" s="272"/>
       <c r="H40" s="272"/>
@@ -6378,61 +6378,61 @@
       <c r="L40" s="210"/>
     </row>
     <row r="41" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="436" t="s">
+      <c r="A41" s="406" t="s">
         <v>150</v>
       </c>
-      <c r="B41" s="437"/>
-      <c r="C41" s="438"/>
-      <c r="D41" s="436"/>
-      <c r="E41" s="438"/>
+      <c r="B41" s="407"/>
+      <c r="C41" s="408"/>
+      <c r="D41" s="406"/>
+      <c r="E41" s="408"/>
       <c r="F41" s="221"/>
       <c r="K41" s="210"/>
       <c r="L41" s="210"/>
     </row>
     <row r="42" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="440" t="s">
+      <c r="A42" s="410" t="s">
         <v>151</v>
       </c>
-      <c r="B42" s="441"/>
-      <c r="C42" s="442"/>
-      <c r="D42" s="436"/>
-      <c r="E42" s="438"/>
+      <c r="B42" s="411"/>
+      <c r="C42" s="412"/>
+      <c r="D42" s="406"/>
+      <c r="E42" s="408"/>
       <c r="F42" s="221"/>
       <c r="K42" s="210"/>
       <c r="L42" s="210"/>
     </row>
     <row r="43" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="440" t="s">
+      <c r="A43" s="410" t="s">
         <v>152</v>
       </c>
-      <c r="B43" s="441"/>
-      <c r="C43" s="442"/>
-      <c r="D43" s="436"/>
-      <c r="E43" s="438"/>
+      <c r="B43" s="411"/>
+      <c r="C43" s="412"/>
+      <c r="D43" s="406"/>
+      <c r="E43" s="408"/>
       <c r="F43" s="221"/>
       <c r="K43" s="210"/>
       <c r="L43" s="210"/>
     </row>
     <row r="44" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="436" t="s">
+      <c r="A44" s="406" t="s">
         <v>153</v>
       </c>
-      <c r="B44" s="437"/>
-      <c r="C44" s="438"/>
-      <c r="D44" s="436"/>
-      <c r="E44" s="438"/>
+      <c r="B44" s="407"/>
+      <c r="C44" s="408"/>
+      <c r="D44" s="406"/>
+      <c r="E44" s="408"/>
       <c r="F44" s="221"/>
       <c r="K44" s="210"/>
       <c r="L44" s="210"/>
     </row>
     <row r="45" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="436" t="s">
+      <c r="A45" s="406" t="s">
         <v>154</v>
       </c>
-      <c r="B45" s="437"/>
-      <c r="C45" s="438"/>
-      <c r="D45" s="436"/>
-      <c r="E45" s="438"/>
+      <c r="B45" s="407"/>
+      <c r="C45" s="408"/>
+      <c r="D45" s="406"/>
+      <c r="E45" s="408"/>
       <c r="F45" s="221"/>
       <c r="K45" s="210"/>
       <c r="L45" s="210"/>
@@ -6525,18 +6525,18 @@
     </row>
     <row r="53" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="54" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="439" t="s">
+      <c r="A54" s="409" t="s">
         <v>170</v>
       </c>
-      <c r="B54" s="439"/>
-      <c r="C54" s="439"/>
-      <c r="D54" s="439"/>
-      <c r="E54" s="439"/>
-      <c r="F54" s="439"/>
-      <c r="G54" s="439"/>
-      <c r="H54" s="439"/>
-      <c r="I54" s="439"/>
-      <c r="J54" s="439"/>
+      <c r="B54" s="409"/>
+      <c r="C54" s="409"/>
+      <c r="D54" s="409"/>
+      <c r="E54" s="409"/>
+      <c r="F54" s="409"/>
+      <c r="G54" s="409"/>
+      <c r="H54" s="409"/>
+      <c r="I54" s="409"/>
+      <c r="J54" s="409"/>
     </row>
     <row r="55" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:12" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -6548,33 +6548,6 @@
     <protectedRange sqref="H31:J31" name="Rango8_1"/>
   </protectedRanges>
   <mergeCells count="39">
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="A54:J54"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="B20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="I16:I18"/>
-    <mergeCell ref="J16:J18"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="A7:J7"/>
     <mergeCell ref="A8:J8"/>
@@ -6587,6 +6560,33 @@
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="A13:J13"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J16:J18"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="A54:J54"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="D44:E44"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0" bottom="0" header="0" footer="0"/>
@@ -6637,38 +6637,38 @@
       <c r="M1" s="295"/>
     </row>
     <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="443" t="s">
+      <c r="A2" s="464" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="443"/>
-      <c r="C2" s="443"/>
-      <c r="D2" s="443"/>
-      <c r="E2" s="443"/>
-      <c r="F2" s="443"/>
-      <c r="G2" s="443"/>
-      <c r="H2" s="443"/>
-      <c r="I2" s="443"/>
-      <c r="J2" s="443"/>
-      <c r="K2" s="443"/>
-      <c r="L2" s="443"/>
-      <c r="M2" s="443"/>
+      <c r="B2" s="464"/>
+      <c r="C2" s="464"/>
+      <c r="D2" s="464"/>
+      <c r="E2" s="464"/>
+      <c r="F2" s="464"/>
+      <c r="G2" s="464"/>
+      <c r="H2" s="464"/>
+      <c r="I2" s="464"/>
+      <c r="J2" s="464"/>
+      <c r="K2" s="464"/>
+      <c r="L2" s="464"/>
+      <c r="M2" s="464"/>
     </row>
     <row r="3" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="444">
+      <c r="A3" s="465">
         <v>0</v>
       </c>
-      <c r="B3" s="444"/>
-      <c r="C3" s="444"/>
-      <c r="D3" s="444"/>
-      <c r="E3" s="444"/>
-      <c r="F3" s="444"/>
-      <c r="G3" s="444"/>
-      <c r="H3" s="444"/>
-      <c r="I3" s="444"/>
-      <c r="J3" s="444"/>
-      <c r="K3" s="444"/>
-      <c r="L3" s="444"/>
-      <c r="M3" s="444"/>
+      <c r="B3" s="465"/>
+      <c r="C3" s="465"/>
+      <c r="D3" s="465"/>
+      <c r="E3" s="465"/>
+      <c r="F3" s="465"/>
+      <c r="G3" s="465"/>
+      <c r="H3" s="465"/>
+      <c r="I3" s="465"/>
+      <c r="J3" s="465"/>
+      <c r="K3" s="465"/>
+      <c r="L3" s="465"/>
+      <c r="M3" s="465"/>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6678,17 +6678,17 @@
       <c r="B5" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="455">
+      <c r="C5" s="476">
         <f>+FORMATO!N2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="455"/>
-      <c r="E5" s="455"/>
-      <c r="F5" s="455"/>
-      <c r="G5" s="455"/>
-      <c r="H5" s="455"/>
-      <c r="I5" s="455"/>
-      <c r="J5" s="455"/>
+      <c r="D5" s="476"/>
+      <c r="E5" s="476"/>
+      <c r="F5" s="476"/>
+      <c r="G5" s="476"/>
+      <c r="H5" s="476"/>
+      <c r="I5" s="476"/>
+      <c r="J5" s="476"/>
       <c r="K5" s="299" t="s">
         <v>20</v>
       </c>
@@ -6706,17 +6706,17 @@
       <c r="B6" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="455">
+      <c r="C6" s="476">
         <f>+FORMATO!N3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="455"/>
-      <c r="E6" s="455"/>
-      <c r="F6" s="455"/>
-      <c r="G6" s="455"/>
-      <c r="H6" s="455"/>
-      <c r="I6" s="455"/>
-      <c r="J6" s="455"/>
+      <c r="D6" s="476"/>
+      <c r="E6" s="476"/>
+      <c r="F6" s="476"/>
+      <c r="G6" s="476"/>
+      <c r="H6" s="476"/>
+      <c r="I6" s="476"/>
+      <c r="J6" s="476"/>
       <c r="K6" s="279" t="s">
         <v>119</v>
       </c>
@@ -6738,17 +6738,17 @@
       <c r="B7" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="455">
+      <c r="C7" s="476">
         <f>+FORMATO!N4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="455"/>
-      <c r="E7" s="455"/>
-      <c r="F7" s="455"/>
-      <c r="G7" s="455"/>
-      <c r="H7" s="455"/>
-      <c r="I7" s="455"/>
-      <c r="J7" s="455"/>
+      <c r="D7" s="476"/>
+      <c r="E7" s="476"/>
+      <c r="F7" s="476"/>
+      <c r="G7" s="476"/>
+      <c r="H7" s="476"/>
+      <c r="I7" s="476"/>
+      <c r="J7" s="476"/>
       <c r="K7" s="279" t="s">
         <v>158</v>
       </c>
@@ -6770,17 +6770,17 @@
       <c r="B8" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="455">
+      <c r="C8" s="476">
         <f>+FORMATO!N5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="455"/>
-      <c r="E8" s="455"/>
-      <c r="F8" s="455"/>
-      <c r="G8" s="455"/>
-      <c r="H8" s="455"/>
-      <c r="I8" s="455"/>
-      <c r="J8" s="455"/>
+      <c r="D8" s="476"/>
+      <c r="E8" s="476"/>
+      <c r="F8" s="476"/>
+      <c r="G8" s="476"/>
+      <c r="H8" s="476"/>
+      <c r="I8" s="476"/>
+      <c r="J8" s="476"/>
       <c r="K8" s="304" t="s">
         <v>36</v>
       </c>
@@ -6816,41 +6816,41 @@
       <c r="P9" s="303"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="447" t="s">
+      <c r="A10" s="468" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="448"/>
-      <c r="C10" s="448"/>
-      <c r="D10" s="448"/>
-      <c r="E10" s="448"/>
-      <c r="F10" s="448"/>
-      <c r="G10" s="448"/>
-      <c r="H10" s="448"/>
-      <c r="I10" s="448"/>
-      <c r="J10" s="448"/>
-      <c r="K10" s="448"/>
-      <c r="L10" s="448"/>
-      <c r="M10" s="449"/>
+      <c r="B10" s="469"/>
+      <c r="C10" s="469"/>
+      <c r="D10" s="469"/>
+      <c r="E10" s="469"/>
+      <c r="F10" s="469"/>
+      <c r="G10" s="469"/>
+      <c r="H10" s="469"/>
+      <c r="I10" s="469"/>
+      <c r="J10" s="469"/>
+      <c r="K10" s="469"/>
+      <c r="L10" s="469"/>
+      <c r="M10" s="470"/>
       <c r="N10" s="303"/>
       <c r="O10" s="303"/>
       <c r="P10" s="303"/>
     </row>
     <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="450" t="s">
+      <c r="A11" s="471" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="451"/>
-      <c r="C11" s="451"/>
-      <c r="D11" s="451"/>
-      <c r="E11" s="451"/>
-      <c r="F11" s="451"/>
-      <c r="G11" s="451"/>
-      <c r="H11" s="451"/>
-      <c r="I11" s="451"/>
-      <c r="J11" s="451"/>
-      <c r="K11" s="451"/>
-      <c r="L11" s="451"/>
-      <c r="M11" s="452"/>
+      <c r="B11" s="472"/>
+      <c r="C11" s="472"/>
+      <c r="D11" s="472"/>
+      <c r="E11" s="472"/>
+      <c r="F11" s="472"/>
+      <c r="G11" s="472"/>
+      <c r="H11" s="472"/>
+      <c r="I11" s="472"/>
+      <c r="J11" s="472"/>
+      <c r="K11" s="472"/>
+      <c r="L11" s="472"/>
+      <c r="M11" s="473"/>
       <c r="N11" s="303"/>
       <c r="O11" s="303"/>
       <c r="P11" s="303"/>
@@ -6874,13 +6874,13 @@
       <c r="P12" s="303"/>
     </row>
     <row r="13" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="453" t="s">
+      <c r="A13" s="474" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="454"/>
-      <c r="C13" s="454"/>
-      <c r="D13" s="454"/>
-      <c r="E13" s="454"/>
+      <c r="B13" s="475"/>
+      <c r="C13" s="475"/>
+      <c r="D13" s="475"/>
+      <c r="E13" s="475"/>
       <c r="F13" s="318"/>
       <c r="G13" s="318"/>
       <c r="H13" s="318"/>
@@ -7011,15 +7011,15 @@
       <c r="A18" s="341"/>
       <c r="B18" s="342"/>
       <c r="C18" s="342"/>
-      <c r="D18" s="445"/>
-      <c r="E18" s="445"/>
+      <c r="D18" s="466"/>
+      <c r="E18" s="466"/>
       <c r="F18" s="342"/>
       <c r="G18" s="342"/>
       <c r="H18" s="342"/>
       <c r="I18" s="343"/>
       <c r="J18" s="343"/>
-      <c r="K18" s="446"/>
-      <c r="L18" s="446"/>
+      <c r="K18" s="467"/>
+      <c r="L18" s="467"/>
       <c r="M18" s="344"/>
       <c r="N18" s="303"/>
       <c r="O18" s="345"/>
@@ -7029,18 +7029,18 @@
       <c r="A19" s="346"/>
       <c r="B19" s="347"/>
       <c r="C19" s="347"/>
-      <c r="D19" s="456" t="s">
+      <c r="D19" s="443" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="457"/>
-      <c r="F19" s="457"/>
-      <c r="G19" s="457"/>
-      <c r="H19" s="458"/>
-      <c r="I19" s="474" t="s">
+      <c r="E19" s="444"/>
+      <c r="F19" s="444"/>
+      <c r="G19" s="444"/>
+      <c r="H19" s="445"/>
+      <c r="I19" s="461" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="474"/>
-      <c r="K19" s="475"/>
+      <c r="J19" s="461"/>
+      <c r="K19" s="462"/>
       <c r="L19" s="348"/>
       <c r="M19" s="349"/>
       <c r="N19" s="303"/>
@@ -7051,11 +7051,11 @@
       <c r="A20" s="350"/>
       <c r="B20" s="295"/>
       <c r="C20" s="295"/>
-      <c r="D20" s="459"/>
-      <c r="E20" s="460"/>
-      <c r="F20" s="460"/>
-      <c r="G20" s="460"/>
-      <c r="H20" s="461"/>
+      <c r="D20" s="446"/>
+      <c r="E20" s="447"/>
+      <c r="F20" s="447"/>
+      <c r="G20" s="447"/>
+      <c r="H20" s="448"/>
       <c r="I20" s="351">
         <v>1</v>
       </c>
@@ -7127,8 +7127,8 @@
         <f>+Datos!I14</f>
         <v>0</v>
       </c>
-      <c r="L22" s="468"/>
-      <c r="M22" s="467"/>
+      <c r="L22" s="455"/>
+      <c r="M22" s="454"/>
       <c r="N22" s="303"/>
       <c r="O22" s="364"/>
       <c r="P22" s="303"/>
@@ -7158,8 +7158,8 @@
         <f>+Datos!I15</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="L23" s="466"/>
-      <c r="M23" s="467"/>
+      <c r="L23" s="453"/>
+      <c r="M23" s="454"/>
       <c r="N23" s="303"/>
       <c r="O23" s="303"/>
       <c r="P23" s="364"/>
@@ -7177,12 +7177,12 @@
       <c r="H24" s="360" t="s">
         <v>1</v>
       </c>
-      <c r="I24" s="469" t="e">
+      <c r="I24" s="456" t="e">
         <f>+Datos!G16</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="J24" s="470"/>
-      <c r="K24" s="471"/>
+      <c r="J24" s="457"/>
+      <c r="K24" s="458"/>
       <c r="L24" s="369"/>
       <c r="M24" s="362"/>
       <c r="N24" s="303"/>
@@ -7244,10 +7244,10 @@
       <c r="C28" s="386"/>
       <c r="D28" s="367"/>
       <c r="E28" s="369"/>
-      <c r="F28" s="472" t="s">
+      <c r="F28" s="459" t="s">
         <v>176</v>
       </c>
-      <c r="G28" s="473"/>
+      <c r="G28" s="460"/>
       <c r="M28" s="384"/>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -7270,11 +7270,11 @@
       <c r="C30" s="386"/>
       <c r="D30" s="367"/>
       <c r="E30" s="369"/>
-      <c r="F30" s="462">
+      <c r="F30" s="449">
         <f>+Datos!E25</f>
         <v>0</v>
       </c>
-      <c r="G30" s="463"/>
+      <c r="G30" s="450"/>
       <c r="M30" s="384"/>
     </row>
     <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -7285,11 +7285,11 @@
       <c r="C31" s="386"/>
       <c r="D31" s="367"/>
       <c r="E31" s="369"/>
-      <c r="F31" s="462">
+      <c r="F31" s="449">
         <f>+Datos!E26</f>
         <v>0</v>
       </c>
-      <c r="G31" s="463"/>
+      <c r="G31" s="450"/>
       <c r="M31" s="384"/>
     </row>
     <row r="32" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -7326,95 +7326,95 @@
       <c r="M34" s="393"/>
     </row>
     <row r="35" spans="1:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="476" t="s">
+      <c r="A35" s="463" t="s">
         <v>171</v>
       </c>
-      <c r="B35" s="476"/>
-      <c r="C35" s="476"/>
-      <c r="D35" s="476"/>
-      <c r="E35" s="476"/>
-      <c r="F35" s="476"/>
-      <c r="G35" s="476"/>
-      <c r="H35" s="476"/>
-      <c r="I35" s="476"/>
-      <c r="J35" s="476"/>
-      <c r="K35" s="476"/>
-      <c r="L35" s="476"/>
-      <c r="M35" s="476"/>
+      <c r="B35" s="463"/>
+      <c r="C35" s="463"/>
+      <c r="D35" s="463"/>
+      <c r="E35" s="463"/>
+      <c r="F35" s="463"/>
+      <c r="G35" s="463"/>
+      <c r="H35" s="463"/>
+      <c r="I35" s="463"/>
+      <c r="J35" s="463"/>
+      <c r="K35" s="463"/>
+      <c r="L35" s="463"/>
+      <c r="M35" s="463"/>
     </row>
     <row r="36" spans="1:16" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="465" t="s">
+      <c r="A36" s="452" t="s">
         <v>172</v>
       </c>
-      <c r="B36" s="465"/>
-      <c r="C36" s="465"/>
-      <c r="D36" s="465"/>
-      <c r="E36" s="465"/>
-      <c r="F36" s="465"/>
-      <c r="G36" s="465"/>
-      <c r="H36" s="465"/>
-      <c r="I36" s="465"/>
-      <c r="J36" s="465"/>
-      <c r="K36" s="465"/>
-      <c r="L36" s="465"/>
-      <c r="M36" s="465"/>
+      <c r="B36" s="452"/>
+      <c r="C36" s="452"/>
+      <c r="D36" s="452"/>
+      <c r="E36" s="452"/>
+      <c r="F36" s="452"/>
+      <c r="G36" s="452"/>
+      <c r="H36" s="452"/>
+      <c r="I36" s="452"/>
+      <c r="J36" s="452"/>
+      <c r="K36" s="452"/>
+      <c r="L36" s="452"/>
+      <c r="M36" s="452"/>
     </row>
     <row r="37" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="465" t="s">
+      <c r="A37" s="452" t="s">
         <v>173</v>
       </c>
-      <c r="B37" s="465"/>
-      <c r="C37" s="465"/>
-      <c r="D37" s="465"/>
-      <c r="E37" s="465"/>
-      <c r="F37" s="465"/>
-      <c r="G37" s="465"/>
-      <c r="H37" s="465"/>
-      <c r="I37" s="465"/>
-      <c r="J37" s="465"/>
-      <c r="K37" s="465"/>
-      <c r="L37" s="465"/>
-      <c r="M37" s="465"/>
+      <c r="B37" s="452"/>
+      <c r="C37" s="452"/>
+      <c r="D37" s="452"/>
+      <c r="E37" s="452"/>
+      <c r="F37" s="452"/>
+      <c r="G37" s="452"/>
+      <c r="H37" s="452"/>
+      <c r="I37" s="452"/>
+      <c r="J37" s="452"/>
+      <c r="K37" s="452"/>
+      <c r="L37" s="452"/>
+      <c r="M37" s="452"/>
       <c r="N37" s="303"/>
       <c r="O37" s="303"/>
       <c r="P37" s="303"/>
     </row>
     <row r="38" spans="1:16" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="465" t="s">
+      <c r="A38" s="452" t="s">
         <v>174</v>
       </c>
-      <c r="B38" s="465"/>
-      <c r="C38" s="465"/>
-      <c r="D38" s="465"/>
-      <c r="E38" s="465"/>
-      <c r="F38" s="465"/>
-      <c r="G38" s="465"/>
-      <c r="H38" s="465"/>
-      <c r="I38" s="465"/>
-      <c r="J38" s="465"/>
-      <c r="K38" s="465"/>
-      <c r="L38" s="465"/>
-      <c r="M38" s="465"/>
+      <c r="B38" s="452"/>
+      <c r="C38" s="452"/>
+      <c r="D38" s="452"/>
+      <c r="E38" s="452"/>
+      <c r="F38" s="452"/>
+      <c r="G38" s="452"/>
+      <c r="H38" s="452"/>
+      <c r="I38" s="452"/>
+      <c r="J38" s="452"/>
+      <c r="K38" s="452"/>
+      <c r="L38" s="452"/>
+      <c r="M38" s="452"/>
       <c r="N38" s="303"/>
       <c r="O38" s="303"/>
       <c r="P38" s="303"/>
     </row>
     <row r="39" spans="1:16" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="464" t="s">
+      <c r="A39" s="451" t="s">
         <v>175</v>
       </c>
-      <c r="B39" s="464"/>
-      <c r="C39" s="464"/>
-      <c r="D39" s="464"/>
-      <c r="E39" s="464"/>
-      <c r="F39" s="464"/>
-      <c r="G39" s="464"/>
-      <c r="H39" s="464"/>
-      <c r="I39" s="464"/>
-      <c r="J39" s="464"/>
-      <c r="K39" s="464"/>
-      <c r="L39" s="464"/>
-      <c r="M39" s="464"/>
+      <c r="B39" s="451"/>
+      <c r="C39" s="451"/>
+      <c r="D39" s="451"/>
+      <c r="E39" s="451"/>
+      <c r="F39" s="451"/>
+      <c r="G39" s="451"/>
+      <c r="H39" s="451"/>
+      <c r="I39" s="451"/>
+      <c r="J39" s="451"/>
+      <c r="K39" s="451"/>
+      <c r="L39" s="451"/>
+      <c r="M39" s="451"/>
       <c r="N39" s="303"/>
       <c r="O39" s="303"/>
       <c r="P39" s="303"/>
@@ -7612,13 +7612,24 @@
     </row>
     <row r="51" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="8NM1+p6p3LesDUstMxFGHu0zYxm1d4zXGYtLxhJOWwI+xJ9//NVS0q83GcKW2Ki+XgVMpMuspxvNsKuxOQLOxg==" saltValue="QYjBUm0XnOsAQh3sj8wCVA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
     <protectedRange sqref="E12" name="Rango3_3_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="E7:E9 C7:D8" name="Rango3_3_1_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="C5:E6" name="Rango3_3_1_1_1_1_1_2_1_1"/>
   </protectedRanges>
   <mergeCells count="24">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="A10:M10"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C8:J8"/>
     <mergeCell ref="D19:H20"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F31:G31"/>
@@ -7632,19 +7643,8 @@
     <mergeCell ref="A35:M35"/>
     <mergeCell ref="A36:M36"/>
     <mergeCell ref="A38:M38"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="A10:M10"/>
-    <mergeCell ref="A11:M11"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="C6:J6"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C8:J8"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F28:G28" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"-,Procedimiento A,Procedimiento B"</formula1>
     </dataValidation>
@@ -7653,7 +7653,7 @@
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0" right="0" top="1.3779527559055118" bottom="0" header="0.11811023622047245" footer="0"/>
+  <pageMargins left="0" right="0" top="1.3779527559055118" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="274" scale="90" orientation="portrait" r:id="rId1"/>
   <headerFooter scaleWithDoc="0">
     <oddHeader>&amp;C&amp;G</oddHeader>

</xml_diff>